<commit_message>
Updates output files with new variant
</commit_message>
<xml_diff>
--- a/Project Outputs for UZ_D_Voltage/Rev04/BOM/BOM_UZ_D_Voltage_3V3_to_3V3_IO.xlsx
+++ b/Project Outputs for UZ_D_Voltage/Rev04/BOM/BOM_UZ_D_Voltage_3V3_to_3V3_IO.xlsx
@@ -1,28 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24228"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Thilo Wendt\Documents\altium\uz_d_voltage\Project Outputs for UZ_D_Voltage\Rev04\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\UltraZohm\uz_d_voltage\Project Outputs for UZ_D_Voltage\Rev04\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DD13D386-ECF8-4456-8C47-AAC08FC2DF04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{74F9736B-97B9-4C73-B5E9-3C09D58C9056}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8964" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3840" yWindow="3840" windowWidth="23040" windowHeight="12060" xr2:uid="{C710180A-45EC-4E7A-8161-1F7564C0BFA6}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="BOM_UZ_D_Voltage_3V3_to_3V3_IO" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">BOM_UZ_D_Voltage_3V3_to_3V3_IO!$1:$1</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
         <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -30,113 +39,160 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="47">
+  <si>
+    <t>Line #</t>
+  </si>
   <si>
     <t>Comment</t>
   </si>
   <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Designator</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>Manufacturer 1</t>
+  </si>
+  <si>
+    <t>Manufacturer Part Number 1</t>
+  </si>
+  <si>
+    <t>Manufacturer Lifecycle 1</t>
+  </si>
+  <si>
+    <t>Supplier 1</t>
+  </si>
+  <si>
+    <t>Supplier Part Number 1</t>
+  </si>
+  <si>
+    <t>Supplier Unit Price 1</t>
+  </si>
+  <si>
+    <t>Supplier Subtotal 1</t>
+  </si>
+  <si>
+    <t>LED ORANGE 600~610NM 80~220MCD@20MA TOP VIEW 0603 ROHS</t>
+  </si>
+  <si>
+    <t>D1</t>
+  </si>
+  <si>
+    <t>LCSC</t>
+  </si>
+  <si>
+    <t>#NAME?</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>0R</t>
   </si>
   <si>
+    <t>SMD resistor E24 series</t>
+  </si>
+  <si>
+    <t>R1, R3A, R3B, R3C, R3D, R3E, R4A, R4B, R4C, R4D, R4E, R5A, R5B, R5C, R5D, R5E, R6A, R6B, R6C, R6D, R6E, R7A, R7B, R7C, R7D, R7E, R8A, R8B, R8C, R8D, R8E, R21, R22, R23, R24, R25, R26, R27, R28, R29, R30, R31, R32, R33, R34, R35, R36, R37, R38, R39, R40, R41, R42, R43, R44, R45, R46, R47, R48, R49, R50, R51, R52, R53, R54, R55, R56, R57, R58, R59, R60, R61, R62, R63, R64, R65, R66, R67, R68, R69, R70, R71, R72, R73, R74, R75, R76, R77, R78, R79, R80</t>
+  </si>
+  <si>
+    <t>Uniroyal</t>
+  </si>
+  <si>
+    <t>0603WAF0000T5E</t>
+  </si>
+  <si>
+    <t>Unknown</t>
+  </si>
+  <si>
+    <t>C21189</t>
+  </si>
+  <si>
     <t>470R</t>
   </si>
   <si>
+    <t>R9</t>
+  </si>
+  <si>
+    <t>KOA Speer</t>
+  </si>
+  <si>
+    <t>RK73B1JTTD471J</t>
+  </si>
+  <si>
+    <t>Volume Production</t>
+  </si>
+  <si>
+    <t>Mouser</t>
+  </si>
+  <si>
+    <t>660-RK73B1JTTD471J</t>
+  </si>
+  <si>
     <t>47R</t>
   </si>
   <si>
+    <t>R82, R84, R85, R87, R90, R92, R93, R95, R98, R100, R101, R103, R106, R108, R109, R111, R114, R116, R117, R119, R122, R124, R125, R127, R130, R132, R133, R135, R138, R139</t>
+  </si>
+  <si>
+    <t>0603WAF470JT5E</t>
+  </si>
+  <si>
+    <t>C23182</t>
+  </si>
+  <si>
     <t>39R</t>
   </si>
   <si>
+    <t>R144, R145, R146, R147, R148, R149, R150, R151, R152, R153, R154, R155, R156, R157, R158, R159, R160, R161, R162, R163, R164, R165, R166, R167, R168, R169, R170, R171, R172, R173</t>
+  </si>
+  <si>
+    <t>0603WAF390JT5E</t>
+  </si>
+  <si>
+    <t>C23154</t>
+  </si>
+  <si>
     <t>IPL1-115-01-L-D-RA-K</t>
   </si>
   <si>
+    <t>Terminal Assembly, Double Row, Right Angle, Thru-Hole, 2.54 mm x 2.54 mm Pitch, 30 Pins</t>
+  </si>
+  <si>
+    <t>X2</t>
+  </si>
+  <si>
+    <t>Samtec</t>
+  </si>
+  <si>
     <t>IPL1-120-01-L-D-RA-K</t>
   </si>
   <si>
-    <t>Designator</t>
-  </si>
-  <si>
-    <t>D1</t>
-  </si>
-  <si>
-    <t>R1, R3A, R3B, R3C, R3D, R3E, R4A, R4B, R4C, R4D, R4E, R5A, R5B, R5C, R5D, R5E, R6A, R6B, R6C, R6D, R6E, R7A, R7B, R7C, R7D, R7E, R8A, R8B, R8C, R8D, R8E, R21, R22, R23, R24, R25, R26, R27, R28, R29, R30, R31, R32, R33, R34, R35, R36, R37, R38, R39, R40, R41, R42, R43, R44, R45, R46, R47, R48, R49, R50, R51, R52, R53, R54, R55, R56, R57, R58, R59, R60, R61, R62, R63, R64, R65, R66, R67, R68, R69, R70, R71, R72, R73, R74, R75, R76, R77, R78, R79, R80</t>
-  </si>
-  <si>
-    <t>R9</t>
-  </si>
-  <si>
-    <t>R82, R84, R85, R87, R90, R92, R93, R95, R98, R100, R101, R103, R106, R108, R109, R111, R114, R116, R117, R119, R122, R124, R125, R127, R130, R132, R133, R135, R138, R139</t>
-  </si>
-  <si>
-    <t>R144, R145, R146, R147, R148, R149, R150, R151, R152, R153, R154, R155, R156, R157, R158, R159, R160, R161, R162, R163, R164, R165, R166, R167, R168, R169, R170, R171, R172, R173</t>
-  </si>
-  <si>
-    <t>X2</t>
+    <t>Terminal Assembly, Double Row, Right Angle, Thru-Hole, 2.54 mm x 2.54 mm Pitch, 40 Pins</t>
   </si>
   <si>
     <t>X3</t>
   </si>
   <si>
-    <t>Footprint</t>
-  </si>
-  <si>
-    <t>WL-SMCW_0603</t>
-  </si>
-  <si>
-    <t>RES 0603_1608, RES 0603_1608 NO TO</t>
-  </si>
-  <si>
-    <t>RES 0603_1608</t>
-  </si>
-  <si>
-    <t>IPL1-115-01-XX-D-RA</t>
-  </si>
-  <si>
-    <t>IPL1-120-01-XX-D-RA</t>
-  </si>
-  <si>
-    <t>LCSC Part #</t>
-  </si>
-  <si>
-    <t>C84269</t>
-  </si>
-  <si>
-    <t>C21189</t>
-  </si>
-  <si>
-    <t>C23179</t>
-  </si>
-  <si>
-    <t>C23182</t>
-  </si>
-  <si>
-    <t>C23154</t>
+    <t>SAMTEC</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="134"/>
     </font>
   </fonts>
   <fills count="3">
@@ -148,7 +204,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor rgb="FFD3D3D3"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -163,41 +219,29 @@
     </border>
     <border>
       <left style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </left>
       <right style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </right>
       <top style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="5">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -226,44 +270,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="0E2841"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="E8E8E8"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="156082"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="E97132"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="196B24"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="0F9ED5"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="A02B93"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="4EA72E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="467886"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="96607D"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light"/>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hans" typeface="等线 Light"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -291,14 +335,31 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hans" typeface="等线"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -326,6 +387,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -387,13 +465,6 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
@@ -402,6 +473,13 @@
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -466,137 +544,342 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+    </a:ext>
+  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B6FC533-1AAA-43B2-A3B0-560CB9BFC048}">
+  <dimension ref="A1:L8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="9.21875" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" customWidth="1"/>
+    <col min="4" max="4" width="13.109375" customWidth="1"/>
+    <col min="5" max="5" width="11.21875" customWidth="1"/>
+    <col min="6" max="6" width="16.44140625" customWidth="1"/>
+    <col min="7" max="7" width="27.21875" customWidth="1"/>
+    <col min="8" max="8" width="23.6640625" customWidth="1"/>
+    <col min="9" max="9" width="12.77734375" customWidth="1"/>
+    <col min="10" max="10" width="23" customWidth="1"/>
+    <col min="11" max="11" width="20.5546875" customWidth="1"/>
+    <col min="12" max="12" width="19.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="I1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="1">
+        <v>1</v>
+      </c>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="1">
+        <v>91</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>21</v>
       </c>
+      <c r="H3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K3" s="1">
+        <v>1.1000000000000001E-3</v>
+      </c>
+      <c r="L3" s="1">
+        <v>0.11</v>
+      </c>
     </row>
-    <row r="2" spans="1:4">
-      <c r="A2" s="2" t="e">
-        <v>#NAME?</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="2" t="s">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="15.9" customHeight="1">
-      <c r="A3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="15.9" customHeight="1">
-      <c r="A4" s="2" t="s">
-        <v>2</v>
-      </c>
       <c r="B4" s="2" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="E4" s="1">
+        <v>1</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="K4" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="L4" s="1">
+        <v>0.1</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="15.9" customHeight="1">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>11</v>
+        <v>16</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>25</v>
+        <v>32</v>
+      </c>
+      <c r="E5" s="1">
+        <v>30</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="K5" s="1">
+        <v>1E-3</v>
+      </c>
+      <c r="L5" s="1">
+        <v>0.1</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="15.9" customHeight="1">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>26</v>
+        <v>36</v>
+      </c>
+      <c r="E6" s="1">
+        <v>30</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="K6" s="1">
+        <v>1E-3</v>
+      </c>
+      <c r="L6" s="1">
+        <v>0.1</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="15.9" customHeight="1">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>13</v>
+        <v>16</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>39</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D7" s="2"/>
+        <v>40</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E7" s="1">
+        <v>1</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="K7" s="1">
+        <v>4.2699999999999996</v>
+      </c>
+      <c r="L7" s="1">
+        <v>4.2699999999999996</v>
+      </c>
     </row>
-    <row r="8" spans="1:4" ht="17.100000000000001" customHeight="1">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>14</v>
+        <v>43</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" s="2"/>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="A9" s="4"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
+        <v>44</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E8" s="1">
+        <v>1</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>